<commit_message>
Quebec sources, and new multi-geojson to single pmtile function.
</commit_message>
<xml_diff>
--- a/data/NCC_Compiled_Tenure_Data_Sources/Blue Carbon - ATL Tenure Data.xlsx
+++ b/data/NCC_Compiled_Tenure_Data_Sources/Blue Carbon - ATL Tenure Data.xlsx
@@ -1216,8 +1216,8 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010023058B3D7F88F54B8F614B4819A3D2C3" ma:contentTypeVersion="20" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="6e532cb5723e67282d1dbbae94493ff1">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c44aea68-f73b-45d5-b042-7c498dcb23dc" xmlns:ns3="634edf18-62ba-46f2-a3a7-063d8fb172d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="6d34ce002620c796e605c4c6381de2f5" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010023058B3D7F88F54B8F614B4819A3D2C3" ma:contentTypeVersion="20" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="9c95790c7176aca22ec34ce72732b57f">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="c44aea68-f73b-45d5-b042-7c498dcb23dc" xmlns:ns3="634edf18-62ba-46f2-a3a7-063d8fb172d8" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="25574f8a6590de80ee0d3b5e25636fa8" ns2:_="" ns3:_="">
     <xsd:import namespace="c44aea68-f73b-45d5-b042-7c498dcb23dc"/>
     <xsd:import namespace="634edf18-62ba-46f2-a3a7-063d8fb172d8"/>
     <xsd:element name="properties">
@@ -1251,7 +1251,7 @@
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:dms="http://schemas.microsoft.com/office/2006/documentManagement/types" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls" targetNamespace="c44aea68-f73b-45d5-b042-7c498dcb23dc" elementFormDefault="qualified">
     <xsd:import namespace="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
     <xsd:import namespace="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <xsd:element name="SharedWithUsers" ma:index="8" nillable="true" ma:displayName="Shared With" ma:internalName="SharedWithUsers" ma:readOnly="true">
+    <xsd:element name="SharedWithUsers" ma:index="8" nillable="true" ma:displayName="Partagé avec" ma:internalName="SharedWithUsers" ma:readOnly="true">
       <xsd:complexType>
         <xsd:complexContent>
           <xsd:extension base="dms:UserMulti">
@@ -1270,7 +1270,7 @@
         </xsd:complexContent>
       </xsd:complexType>
     </xsd:element>
-    <xsd:element name="SharedWithDetails" ma:index="9" nillable="true" ma:displayName="Shared With Details" ma:internalName="SharedWithDetails" ma:readOnly="true">
+    <xsd:element name="SharedWithDetails" ma:index="9" nillable="true" ma:displayName="Partagé avec détails" ma:internalName="SharedWithDetails" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Note">
           <xsd:maxLength value="255"/>
@@ -1319,7 +1319,7 @@
         <xsd:restriction base="dms:Text"/>
       </xsd:simpleType>
     </xsd:element>
-    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="17" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Image Tags" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="2baaf764-73f0-4b4c-b8e1-b7d465e0804e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
+    <xsd:element name="lcf76f155ced4ddcb4097134ff3c332f" ma:index="17" nillable="true" ma:taxonomy="true" ma:internalName="lcf76f155ced4ddcb4097134ff3c332f" ma:taxonomyFieldName="MediaServiceImageTags" ma:displayName="Balises d’images" ma:readOnly="false" ma:fieldId="{5cf76f15-5ced-4ddc-b409-7134ff3c332f}" ma:taxonomyMulti="true" ma:sspId="2baaf764-73f0-4b4c-b8e1-b7d465e0804e" ma:termSetId="09814cd3-568e-fe90-9814-8d621ff8fb84" ma:anchorId="fba54fb3-c3e1-fe81-a776-ca4b69148c4d" ma:open="true" ma:isKeyword="false">
       <xsd:complexType>
         <xsd:sequence>
           <xsd:element ref="pc:Terms" minOccurs="0" maxOccurs="1"/>
@@ -1366,8 +1366,8 @@
         <xsd:element ref="dc:creator" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dcterms:created" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:identifier" minOccurs="0" maxOccurs="1"/>
-        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Content Type"/>
-        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Title"/>
+        <xsd:element name="contentType" minOccurs="0" maxOccurs="1" type="xsd:string" ma:index="0" ma:displayName="Type de contenu"/>
+        <xsd:element ref="dc:title" minOccurs="0" maxOccurs="1" ma:index="4" ma:displayName="Titre"/>
         <xsd:element ref="dc:subject" minOccurs="0" maxOccurs="1"/>
         <xsd:element ref="dc:description" minOccurs="0" maxOccurs="1"/>
         <xsd:element name="keywords" minOccurs="0" maxOccurs="1" type="xsd:string"/>
@@ -1476,5 +1476,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{2756C475-5299-4C09-BC2B-B90B2E8912D5}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F43A0BA5-AA28-4826-BA86-088112381C82}"/>
 </file>
</xml_diff>